<commit_message>
✨I can do it
</commit_message>
<xml_diff>
--- a/src/main/resources/许愿墙.xlsx
+++ b/src/main/resources/许愿墙.xlsx
@@ -1,360 +1,86 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{00000000-0001-0000-0000-000000000000}" mc:Ignorable="x14ac xr xr2 xr3 xr6 xr10 x15">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11208"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\project\get_jobs\src\main\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C9FB88-1988-487B-8181-01C1809F3C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowHeight="15800" windowWidth="28040" xWindow="4240" yWindow="640"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcMode="auto"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>你想找什么样的工作？</t>
-  </si>
-  <si>
-    <t>现在的状态是怎样的？</t>
-  </si>
-  <si>
-    <t>AI攻城狮</t>
-  </si>
-  <si>
-    <t>已找到！</t>
-  </si>
-  <si>
-    <t>Java+AI</t>
-  </si>
-  <si>
-    <t>在找</t>
-  </si>
-  <si>
-    <t>AI agent开发</t>
-  </si>
-  <si>
-    <t>Java实习</t>
-  </si>
-  <si>
-    <t>还没开始找</t>
-  </si>
-  <si>
-    <t>系统架构师</t>
-  </si>
-  <si>
-    <t>Go</t>
-  </si>
-  <si>
-    <t>前端攻城狮</t>
-  </si>
-  <si>
-    <t>AI+游戏开发</t>
-  </si>
-  <si>
-    <t>C++实习</t>
-  </si>
-  <si>
-    <t>后端开发</t>
-  </si>
-  <si>
-    <t>正确的路上</t>
-  </si>
-  <si>
-    <t>Java后端开发</t>
-  </si>
-  <si>
-    <t>在找实习的路上</t>
-  </si>
-  <si>
-    <t>Java</t>
-  </si>
-  <si>
-    <t>找到了，但是通勤太远想跳槽</t>
-  </si>
-  <si>
-    <t>Frontend leader</t>
-  </si>
-  <si>
-    <t>找到了，但是没有work life balance</t>
-  </si>
-  <si>
-    <t>找到了，不满意</t>
-  </si>
-  <si>
-    <t>Java开发</t>
-  </si>
-  <si>
-    <t>再找</t>
-  </si>
-  <si>
-    <t>前端工程师</t>
-  </si>
-  <si>
-    <t>java开发</t>
-  </si>
-  <si>
-    <t>AI+前端工程师</t>
-  </si>
-  <si>
-    <t>C++开发</t>
-  </si>
-  <si>
-    <t>Go后端开发</t>
-  </si>
-  <si>
-    <t>AI+后端工程师</t>
-  </si>
-  <si>
-    <t>linux运维</t>
-  </si>
-  <si>
-    <t>AI+嵌入式</t>
-  </si>
-  <si>
-    <t>财务主管</t>
-  </si>
-  <si>
-    <t>在学习的路上</t>
-  </si>
-  <si>
-    <t>去年7月用这个项目找到了第一份工作，现在再次回来，希望跳槽找一份AI售前的工作</t>
-  </si>
-  <si>
-    <t>准备跳槽</t>
-  </si>
-  <si>
-    <t>Java开发，有完善的晋升制度</t>
-  </si>
-  <si>
-    <t>前端开发</t>
-  </si>
-  <si>
-    <t>找到了，兄弟们加油。对于前端这块简历一定要吹牛逼写好，
-面试前真的要背好八股和场景，或者找不想去的公司练练手，准备好了之后再冲刺</t>
-  </si>
-  <si>
-    <t>正在找</t>
-  </si>
-  <si>
-    <t>C#开发</t>
-  </si>
-  <si>
-    <t>dotnet开发，base 成都</t>
-  </si>
-  <si>
-    <t>JAVA开发，base太原</t>
-  </si>
-  <si>
-    <t>前端开发，base上海</t>
-  </si>
-  <si>
-    <t>测试开发</t>
-  </si>
-  <si>
-    <t>运维开发</t>
-  </si>
-  <si>
-    <t>找到了，要去当牛马了，后续准备做独立开发</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 渗透测试工程师</t>
-  </si>
-  <si>
-    <t>应届在找</t>
-  </si>
-  <si>
-    <t>IT审计/数据分析/财务BP</t>
-  </si>
-  <si>
-    <t>AI应用开发</t>
-  </si>
-  <si>
-    <t>设计师</t>
-  </si>
-  <si>
-    <t>Java开发/海外仓销售</t>
-  </si>
-  <si>
-    <t>ai产品</t>
-  </si>
-  <si>
-    <t>数据开发+ai</t>
-  </si>
-  <si>
-    <t>失业了在找</t>
-  </si>
-  <si>
-    <t>AI+JAVA</t>
-  </si>
-  <si>
-    <t>大专，前端工程师，空窗创业，gap一年半😁，找了内推看看机会
-保持学习，看下金九银十有没机会了</t>
-  </si>
-  <si>
-    <t>AI产品</t>
-  </si>
-  <si>
-    <t>Java秋招</t>
-  </si>
-  <si>
-    <t>目前实习，在改简历背八股准备秋招！！！</t>
-  </si>
-  <si>
-    <t>大厂的产品岗_26届秋招</t>
-  </si>
-  <si>
-    <t>应届生正在进行中</t>
-  </si>
-  <si>
-    <t>双休、Java</t>
-  </si>
-  <si>
-    <t>25应届摆烂仔正在行动</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI + JAVA </t>
-  </si>
-  <si>
-    <t>嵌入式Ai</t>
-  </si>
-  <si>
-    <t>全栈架构师 研发经理</t>
-  </si>
-  <si>
-    <t>被裁再找,改好了简历</t>
-  </si>
-  <si>
-    <t>网络安全</t>
-  </si>
-  <si>
-    <t>嵌入式/硬件测试</t>
-  </si>
-  <si>
-    <t>25届毕业生在狂卷</t>
-  </si>
-  <si>
-    <t>Java 中厂</t>
-  </si>
-  <si>
-    <t>刚找到实习，现在边实习边秋招</t>
-  </si>
-  <si>
-    <t>AIGC相关后端或全栈</t>
-  </si>
-  <si>
-    <t>开始找第一天</t>
-  </si>
-  <si>
-    <t>AIGC相关后端或全栈/量化交易员</t>
-  </si>
-  <si>
-    <t>在找，之前上过大厂班，不适应，后续我想做独立开发</t>
-  </si>
-  <si>
-    <t>Java怎么这么难呀（煎熬）</t>
-  </si>
-  <si>
-    <t>数分/AI产品</t>
-  </si>
-  <si>
-    <t>在努力了</t>
-  </si>
-  <si>
-    <t>交互设计</t>
-  </si>
-  <si>
-    <t>在找（好像看下来只有我是学设计的/哭哭）</t>
-  </si>
-  <si>
-    <t>产品经理</t>
-  </si>
-  <si>
-    <t>努力跳槽中</t>
-  </si>
-  <si>
-    <t>数据分析师</t>
-  </si>
-  <si>
-    <t>java高级开发</t>
-  </si>
-  <si>
-    <t>Python后端开发</t>
-  </si>
-  <si>
-    <t>在找，非科班非应届，debuff叠满QAQ</t>
-  </si>
-  <si>
-    <t>AI+java</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>在找了</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9.75"/>
       <color rgb="FF000000"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9.75"/>
       <color rgb="FF000000"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <fgColor/>
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <fgColor/>
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF34C724"/>
+        <bgColor/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -367,21 +93,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF1F2329"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF1F2329"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF1F2329"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF1F2329"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -422,6 +133,34 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1F2329"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F2329"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F2329"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1F2329"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1F2329"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F2329"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F2329"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF1F2329"/>
       </left>
@@ -438,36 +177,39 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="true" applyBorder="false" applyFill="true" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="6" fillId="2" fontId="1" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" applyProtection="false" borderId="7" fillId="0" fontId="1" numFmtId="164" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -480,7 +222,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -775,23 +517,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xr:uid="{00000000-0001-0000-0000-000000000000}" mc:Ignorable="x14ac xr xr2 xr3 xr6 xr10 x15">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <dimension ref="A1:T200"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="19"/>
   <cols>
-    <col min="1" max="1" width="74" customWidth="1"/>
-    <col min="2" max="2" width="75" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="74"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="75"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
+    <row r="1">
+      <c r="A1" s="6" t="str">
+        <v>你想找什么样的工作？</v>
+      </c>
+      <c r="B1" s="6" t="str">
+        <v>现在的状态是怎样的？</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -812,12 +554,12 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
+    <row r="2">
+      <c r="A2" s="4" t="str">
+        <v>财务BP</v>
+      </c>
+      <c r="B2" s="5" t="str">
+        <v>未在找</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -838,12 +580,12 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>财务业务伙伴</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>未在找</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -864,12 +606,12 @@
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>财务控制</v>
+      </c>
+      <c r="B4" s="5" t="str">
+        <v>未在找</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -890,12 +632,12 @@
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
+    <row r="5">
+      <c r="A5" s="2" t="str" xml:space="preserve">
+        <v> JAVA开发</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>正在找</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -916,12 +658,12 @@
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>除了国际短信运营之外的任何</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -942,12 +684,12 @@
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>行政人事，项目助理，写作类的（比如编剧）</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -968,12 +710,12 @@
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>5</v>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>算法C++</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -994,12 +736,12 @@
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>Java开发兼职</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>在找</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1020,12 +762,12 @@
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>5</v>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>Java开发</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>正在找</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1046,12 +788,12 @@
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>15</v>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>CyberSecurity</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1072,12 +814,12 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>17</v>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>数据标注</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1098,12 +840,12 @@
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>19</v>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v>门店运营经理「线下连锁品牌、消费品类」——项目经理「文旅」</v>
+      </c>
+      <c r="B13" s="4" t="str">
+        <v>未在找</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -1124,12 +866,12 @@
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>21</v>
+    <row r="14">
+      <c r="A14" s="4" t="str">
+        <v>运营分析</v>
+      </c>
+      <c r="B14" s="4" t="str">
+        <v>未在找</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1150,12 +892,12 @@
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>22</v>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v>大模型算法</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1176,12 +918,12 @@
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>24</v>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v>海外销售/外企管培/外资银行</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1202,12 +944,12 @@
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>5</v>
+    <row r="17">
+      <c r="A17" s="2" t="str">
+        <v>Java开发</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>在找</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1228,12 +970,12 @@
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>5</v>
+    <row r="18">
+      <c r="A18" s="2" t="str">
+        <v>5年java开发</v>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1254,12 +996,12 @@
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>8</v>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v>产品经理</v>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1280,12 +1022,12 @@
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>5</v>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v>8年前端【远程、线下皆可】</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v>未在找</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1306,12 +1048,12 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>5</v>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v>2026物联网工程师[]</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>在找,找到了就来还愿</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1332,12 +1074,12 @@
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>5</v>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>技术支持 / IT Infra / Azure架构</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>在家躺够了TwT</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1358,12 +1100,12 @@
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>8</v>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>技术支持/软件测试</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>在找</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -1384,12 +1126,12 @@
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>5</v>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>AI应用开发</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>正在找哦（WY）</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -1410,12 +1152,12 @@
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>5</v>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>DBA</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>在学、在找</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1436,12 +1178,12 @@
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>8</v>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>cv算法</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>再找</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -1462,12 +1204,12 @@
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>5</v>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>RAG/python后端开发</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>正在找</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1488,12 +1230,12 @@
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>24</v>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>Java实习</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>正在找,边学边找</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1514,12 +1256,12 @@
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>5</v>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>Java开发实习</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>大四正在找实习</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -1540,12 +1282,12 @@
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>34</v>
+    <row r="30">
+      <c r="A30" s="2" t="str">
+        <v>技术支持/运维/开发</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <v>在职，正在看</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1566,12 +1308,12 @@
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>5</v>
+    <row r="31">
+      <c r="A31" s="2" t="str">
+        <v>我想什么都会做</v>
+      </c>
+      <c r="B31" s="2" t="str">
+        <v>加油</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1592,12 +1334,12 @@
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>5</v>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v>2年前端</v>
+      </c>
+      <c r="B32" s="2" t="str">
+        <v>刚辞职，在找，不知道过年前能不能找到</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1618,12 +1360,12 @@
       <c r="S32" s="1"/>
       <c r="T32" s="1"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>36</v>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v>9年工作经验  5年实施 3年运维 1年前端</v>
+      </c>
+      <c r="B33" s="2" t="str">
+        <v>离职半年了 每天浑浑噩噩 有点颓废 压力又大 近期开始找工作</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1644,12 +1386,12 @@
       <c r="S33" s="1"/>
       <c r="T33" s="1"/>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A34" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>36</v>
+    <row r="34">
+      <c r="A34" s="2" t="str">
+        <v>电离辐射环境咨询人员</v>
+      </c>
+      <c r="B34" s="2" t="str">
+        <v>大四准备面试</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1670,12 +1412,12 @@
       <c r="S34" s="1"/>
       <c r="T34" s="1"/>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A35" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>39</v>
+    <row r="35">
+      <c r="A35" s="2" t="str">
+        <v>AI大模型工程师</v>
+      </c>
+      <c r="B35" s="2" t="str">
+        <v>正在寻找</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1696,12 +1438,12 @@
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>5</v>
+    <row r="36">
+      <c r="A36" s="2" t="str">
+        <v>Java牛马师</v>
+      </c>
+      <c r="B36" s="2" t="str">
+        <v>还在找</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1722,12 +1464,12 @@
       <c r="S36" s="1"/>
       <c r="T36" s="1"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A37" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>40</v>
+    <row r="37">
+      <c r="A37" s="2" t="str">
+        <v>品牌传播、HRBP、运营分析</v>
+      </c>
+      <c r="B37" s="2" t="str">
+        <v>正在找</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -1748,64 +1490,64 @@
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-      <c r="O38" s="1"/>
-      <c r="P38" s="1"/>
-      <c r="Q38" s="1"/>
-      <c r="R38" s="1"/>
-      <c r="S38" s="1"/>
-      <c r="T38" s="1"/>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="4"/>
-      <c r="M39" s="4"/>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
-      <c r="P39" s="4"/>
-      <c r="Q39" s="4"/>
-      <c r="R39" s="4"/>
-      <c r="S39" s="4"/>
-      <c r="T39" s="4"/>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A40" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>5</v>
+    <row r="38">
+      <c r="A38" s="4" t="str">
+        <v>渗透测试工程师、安全服务工程师</v>
+      </c>
+      <c r="B38" s="2" t="str">
+        <v>正在寻找</v>
+      </c>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="3"/>
+      <c r="Q38" s="3"/>
+      <c r="R38" s="3"/>
+      <c r="S38" s="3"/>
+      <c r="T38" s="3"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="str">
+        <v>嵌入式软件工程师</v>
+      </c>
+      <c r="B39" s="2" t="str">
+        <v>还在找</v>
+      </c>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
+      <c r="S39" s="1"/>
+      <c r="T39" s="1"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="str">
+        <v>10年电商运营</v>
+      </c>
+      <c r="B40" s="2" t="str">
+        <v>和之前领导出来创业，公司月底到底，正在寻找工作</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -1826,12 +1568,12 @@
       <c r="S40" s="1"/>
       <c r="T40" s="1"/>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A41" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>5</v>
+    <row r="41">
+      <c r="A41" s="2" t="str">
+        <v>独立摄影师</v>
+      </c>
+      <c r="B41" s="2" t="str">
+        <v>正在学习  各位有想拍照的可以随时联系我</v>
       </c>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
@@ -1852,12 +1594,12 @@
       <c r="S41" s="1"/>
       <c r="T41" s="1"/>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>36</v>
+    <row r="42">
+      <c r="A42" s="2" t="str">
+        <v>java+ai</v>
+      </c>
+      <c r="B42" s="2" t="str">
+        <v>正在跳槽</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -1878,13 +1620,9 @@
       <c r="S42" s="1"/>
       <c r="T42" s="1"/>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="43">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -1904,13 +1642,9 @@
       <c r="S43" s="1"/>
       <c r="T43" s="1"/>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A44" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>36</v>
-      </c>
+    <row r="44">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -1930,13 +1664,9 @@
       <c r="S44" s="1"/>
       <c r="T44" s="1"/>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="45">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -1956,13 +1686,9 @@
       <c r="S45" s="1"/>
       <c r="T45" s="1"/>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="46">
+      <c r="A46" s="7"/>
+      <c r="B46" s="2"/>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -1982,13 +1708,9 @@
       <c r="S46" s="1"/>
       <c r="T46" s="1"/>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A47" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>47</v>
-      </c>
+    <row r="47">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
@@ -2008,13 +1730,9 @@
       <c r="S47" s="1"/>
       <c r="T47" s="1"/>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A48" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>49</v>
-      </c>
+    <row r="48">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
@@ -2034,13 +1752,9 @@
       <c r="S48" s="1"/>
       <c r="T48" s="1"/>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A49" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>36</v>
-      </c>
+    <row r="49">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2060,13 +1774,9 @@
       <c r="S49" s="1"/>
       <c r="T49" s="1"/>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="50">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
@@ -2086,13 +1796,9 @@
       <c r="S50" s="1"/>
       <c r="T50" s="1"/>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A51" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="51">
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
@@ -2112,13 +1818,9 @@
       <c r="S51" s="1"/>
       <c r="T51" s="1"/>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="52">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
@@ -2138,13 +1840,9 @@
       <c r="S52" s="1"/>
       <c r="T52" s="1"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A53" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="53">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
@@ -2164,13 +1862,9 @@
       <c r="S53" s="1"/>
       <c r="T53" s="1"/>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A54" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="54">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
       <c r="C54" s="1"/>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
@@ -2190,13 +1884,9 @@
       <c r="S54" s="1"/>
       <c r="T54" s="1"/>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="55">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
@@ -2216,13 +1906,9 @@
       <c r="S55" s="1"/>
       <c r="T55" s="1"/>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="56">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
@@ -2242,13 +1928,9 @@
       <c r="S56" s="1"/>
       <c r="T56" s="1"/>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>56</v>
-      </c>
+    <row r="57">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
@@ -2268,13 +1950,9 @@
       <c r="S57" s="1"/>
       <c r="T57" s="1"/>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A58" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="58">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
@@ -2294,13 +1972,9 @@
       <c r="S58" s="1"/>
       <c r="T58" s="1"/>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A59" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="59">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
@@ -2320,13 +1994,9 @@
       <c r="S59" s="1"/>
       <c r="T59" s="1"/>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>58</v>
-      </c>
+    <row r="60">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
@@ -2346,13 +2016,9 @@
       <c r="S60" s="1"/>
       <c r="T60" s="1"/>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A61" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="61">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
@@ -2372,13 +2038,9 @@
       <c r="S61" s="1"/>
       <c r="T61" s="1"/>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A62" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>61</v>
-      </c>
+    <row r="62">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
@@ -2398,13 +2060,9 @@
       <c r="S62" s="1"/>
       <c r="T62" s="1"/>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A63" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>63</v>
-      </c>
+    <row r="63">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
@@ -2424,13 +2082,9 @@
       <c r="S63" s="1"/>
       <c r="T63" s="1"/>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A64" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>65</v>
-      </c>
+    <row r="64">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
@@ -2450,13 +2104,9 @@
       <c r="S64" s="1"/>
       <c r="T64" s="1"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A65" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="65">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
@@ -2476,13 +2126,9 @@
       <c r="S65" s="1"/>
       <c r="T65" s="1"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A66" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="66">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
@@ -2502,13 +2148,9 @@
       <c r="S66" s="1"/>
       <c r="T66" s="1"/>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A67" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>69</v>
-      </c>
+    <row r="67">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
@@ -2528,13 +2170,9 @@
       <c r="S67" s="1"/>
       <c r="T67" s="1"/>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A68" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="68">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
@@ -2554,13 +2192,9 @@
       <c r="S68" s="1"/>
       <c r="T68" s="1"/>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A69" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="69">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
@@ -2580,13 +2214,9 @@
       <c r="S69" s="1"/>
       <c r="T69" s="1"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="70">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
@@ -2606,13 +2236,9 @@
       <c r="S70" s="1"/>
       <c r="T70" s="1"/>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="71">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
@@ -2632,13 +2258,9 @@
       <c r="S71" s="1"/>
       <c r="T71" s="1"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A72" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>72</v>
-      </c>
+    <row r="72">
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
@@ -2658,13 +2280,9 @@
       <c r="S72" s="1"/>
       <c r="T72" s="1"/>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>74</v>
-      </c>
+    <row r="73">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
@@ -2684,13 +2302,9 @@
       <c r="S73" s="1"/>
       <c r="T73" s="1"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A74" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="74">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
@@ -2710,13 +2324,9 @@
       <c r="S74" s="1"/>
       <c r="T74" s="1"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A75" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>76</v>
-      </c>
+    <row r="75">
+      <c r="A75" s="3"/>
+      <c r="B75" s="2"/>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
@@ -2736,13 +2346,9 @@
       <c r="S75" s="1"/>
       <c r="T75" s="1"/>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A76" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>78</v>
-      </c>
+    <row r="76">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
@@ -2762,13 +2368,9 @@
       <c r="S76" s="1"/>
       <c r="T76" s="1"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A77" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>79</v>
-      </c>
+    <row r="77">
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
@@ -2788,13 +2390,9 @@
       <c r="S77" s="1"/>
       <c r="T77" s="1"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A78" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>81</v>
-      </c>
+    <row r="78">
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
@@ -2814,13 +2412,9 @@
       <c r="S78" s="1"/>
       <c r="T78" s="1"/>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>83</v>
-      </c>
+    <row r="79">
+      <c r="A79" s="2"/>
+      <c r="B79" s="2"/>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
       <c r="E79" s="1"/>
@@ -2840,13 +2434,9 @@
       <c r="S79" s="1"/>
       <c r="T79" s="1"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A80" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>85</v>
-      </c>
+    <row r="80">
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
       <c r="E80" s="1"/>
@@ -2866,13 +2456,9 @@
       <c r="S80" s="1"/>
       <c r="T80" s="1"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A81" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="81">
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
@@ -2892,13 +2478,9 @@
       <c r="S81" s="1"/>
       <c r="T81" s="1"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A82" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="82">
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
@@ -2918,13 +2500,9 @@
       <c r="S82" s="1"/>
       <c r="T82" s="1"/>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A83" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>89</v>
-      </c>
+    <row r="83">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
       <c r="E83" s="1"/>
@@ -2944,13 +2522,9 @@
       <c r="S83" s="1"/>
       <c r="T83" s="1"/>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A84" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>91</v>
-      </c>
+    <row r="84">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
       <c r="E84" s="1"/>
@@ -2970,7 +2544,7 @@
       <c r="S84" s="1"/>
       <c r="T84" s="1"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="85">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="1"/>
@@ -2992,7 +2566,7 @@
       <c r="S85" s="1"/>
       <c r="T85" s="1"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="86">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="1"/>
@@ -3014,7 +2588,7 @@
       <c r="S86" s="1"/>
       <c r="T86" s="1"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="87">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="1"/>
@@ -3036,7 +2610,7 @@
       <c r="S87" s="1"/>
       <c r="T87" s="1"/>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="88">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="1"/>
@@ -3058,7 +2632,7 @@
       <c r="S88" s="1"/>
       <c r="T88" s="1"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="89">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="1"/>
@@ -3080,7 +2654,7 @@
       <c r="S89" s="1"/>
       <c r="T89" s="1"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="90">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="1"/>
@@ -3102,7 +2676,7 @@
       <c r="S90" s="1"/>
       <c r="T90" s="1"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="91">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="1"/>
@@ -3124,7 +2698,7 @@
       <c r="S91" s="1"/>
       <c r="T91" s="1"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="92">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="1"/>
@@ -3146,7 +2720,7 @@
       <c r="S92" s="1"/>
       <c r="T92" s="1"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="93">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="1"/>
@@ -3168,7 +2742,7 @@
       <c r="S93" s="1"/>
       <c r="T93" s="1"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="94">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="1"/>
@@ -3190,7 +2764,7 @@
       <c r="S94" s="1"/>
       <c r="T94" s="1"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="95">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="1"/>
@@ -3212,7 +2786,7 @@
       <c r="S95" s="1"/>
       <c r="T95" s="1"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="96">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="1"/>
@@ -3234,7 +2808,7 @@
       <c r="S96" s="1"/>
       <c r="T96" s="1"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="97">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="1"/>
@@ -3256,7 +2830,7 @@
       <c r="S97" s="1"/>
       <c r="T97" s="1"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="98">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="1"/>
@@ -3278,7 +2852,7 @@
       <c r="S98" s="1"/>
       <c r="T98" s="1"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="99">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="1"/>
@@ -3300,7 +2874,7 @@
       <c r="S99" s="1"/>
       <c r="T99" s="1"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="100">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="1"/>
@@ -3322,7 +2896,7 @@
       <c r="S100" s="1"/>
       <c r="T100" s="1"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="101">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="1"/>
@@ -3344,7 +2918,7 @@
       <c r="S101" s="1"/>
       <c r="T101" s="1"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="102">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="1"/>
@@ -3366,7 +2940,7 @@
       <c r="S102" s="1"/>
       <c r="T102" s="1"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="103">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="1"/>
@@ -3388,7 +2962,7 @@
       <c r="S103" s="1"/>
       <c r="T103" s="1"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="104">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="1"/>
@@ -3410,7 +2984,7 @@
       <c r="S104" s="1"/>
       <c r="T104" s="1"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="105">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="1"/>
@@ -3432,7 +3006,7 @@
       <c r="S105" s="1"/>
       <c r="T105" s="1"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="106">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="1"/>
@@ -3454,7 +3028,7 @@
       <c r="S106" s="1"/>
       <c r="T106" s="1"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="107">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="1"/>
@@ -3476,7 +3050,7 @@
       <c r="S107" s="1"/>
       <c r="T107" s="1"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="108">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="1"/>
@@ -3498,7 +3072,7 @@
       <c r="S108" s="1"/>
       <c r="T108" s="1"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="109">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="1"/>
@@ -3520,7 +3094,7 @@
       <c r="S109" s="1"/>
       <c r="T109" s="1"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="110">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="1"/>
@@ -3542,7 +3116,7 @@
       <c r="S110" s="1"/>
       <c r="T110" s="1"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="111">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="1"/>
@@ -3564,7 +3138,7 @@
       <c r="S111" s="1"/>
       <c r="T111" s="1"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="112">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="1"/>
@@ -3586,7 +3160,7 @@
       <c r="S112" s="1"/>
       <c r="T112" s="1"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="113">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="1"/>
@@ -3608,7 +3182,7 @@
       <c r="S113" s="1"/>
       <c r="T113" s="1"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="114">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="1"/>
@@ -3630,7 +3204,7 @@
       <c r="S114" s="1"/>
       <c r="T114" s="1"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="115">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="1"/>
@@ -3652,7 +3226,7 @@
       <c r="S115" s="1"/>
       <c r="T115" s="1"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="116">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="1"/>
@@ -3674,7 +3248,7 @@
       <c r="S116" s="1"/>
       <c r="T116" s="1"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="117">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="1"/>
@@ -3696,7 +3270,7 @@
       <c r="S117" s="1"/>
       <c r="T117" s="1"/>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="118">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="1"/>
@@ -3718,7 +3292,7 @@
       <c r="S118" s="1"/>
       <c r="T118" s="1"/>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="119">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="1"/>
@@ -3740,7 +3314,7 @@
       <c r="S119" s="1"/>
       <c r="T119" s="1"/>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="120">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="1"/>
@@ -3762,7 +3336,7 @@
       <c r="S120" s="1"/>
       <c r="T120" s="1"/>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="121">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="1"/>
@@ -3784,7 +3358,7 @@
       <c r="S121" s="1"/>
       <c r="T121" s="1"/>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="122">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="1"/>
@@ -3806,7 +3380,7 @@
       <c r="S122" s="1"/>
       <c r="T122" s="1"/>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="123">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="1"/>
@@ -3828,7 +3402,7 @@
       <c r="S123" s="1"/>
       <c r="T123" s="1"/>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="124">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="1"/>
@@ -3850,7 +3424,7 @@
       <c r="S124" s="1"/>
       <c r="T124" s="1"/>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="125">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="1"/>
@@ -3872,7 +3446,7 @@
       <c r="S125" s="1"/>
       <c r="T125" s="1"/>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="126">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="1"/>
@@ -3894,7 +3468,7 @@
       <c r="S126" s="1"/>
       <c r="T126" s="1"/>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="127">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="1"/>
@@ -3916,7 +3490,7 @@
       <c r="S127" s="1"/>
       <c r="T127" s="1"/>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="128">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="1"/>
@@ -3938,7 +3512,7 @@
       <c r="S128" s="1"/>
       <c r="T128" s="1"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="129">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="1"/>
@@ -3960,7 +3534,7 @@
       <c r="S129" s="1"/>
       <c r="T129" s="1"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="130">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="1"/>
@@ -3982,7 +3556,7 @@
       <c r="S130" s="1"/>
       <c r="T130" s="1"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="131">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="1"/>
@@ -4004,7 +3578,7 @@
       <c r="S131" s="1"/>
       <c r="T131" s="1"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="132">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="1"/>
@@ -4026,7 +3600,7 @@
       <c r="S132" s="1"/>
       <c r="T132" s="1"/>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="133">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="1"/>
@@ -4048,7 +3622,7 @@
       <c r="S133" s="1"/>
       <c r="T133" s="1"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="134">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="1"/>
@@ -4070,7 +3644,7 @@
       <c r="S134" s="1"/>
       <c r="T134" s="1"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="135">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="1"/>
@@ -4092,7 +3666,7 @@
       <c r="S135" s="1"/>
       <c r="T135" s="1"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="136">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="1"/>
@@ -4114,7 +3688,7 @@
       <c r="S136" s="1"/>
       <c r="T136" s="1"/>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="137">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="1"/>
@@ -4136,7 +3710,7 @@
       <c r="S137" s="1"/>
       <c r="T137" s="1"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="138">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="1"/>
@@ -4158,7 +3732,7 @@
       <c r="S138" s="1"/>
       <c r="T138" s="1"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="139">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="1"/>
@@ -4180,7 +3754,7 @@
       <c r="S139" s="1"/>
       <c r="T139" s="1"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="140">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="1"/>
@@ -4202,7 +3776,7 @@
       <c r="S140" s="1"/>
       <c r="T140" s="1"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="141">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="1"/>
@@ -4224,7 +3798,7 @@
       <c r="S141" s="1"/>
       <c r="T141" s="1"/>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="142">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="1"/>
@@ -4246,7 +3820,7 @@
       <c r="S142" s="1"/>
       <c r="T142" s="1"/>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="143">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="1"/>
@@ -4268,7 +3842,7 @@
       <c r="S143" s="1"/>
       <c r="T143" s="1"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="144">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="1"/>
@@ -4290,7 +3864,7 @@
       <c r="S144" s="1"/>
       <c r="T144" s="1"/>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="145">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="1"/>
@@ -4312,7 +3886,7 @@
       <c r="S145" s="1"/>
       <c r="T145" s="1"/>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="146">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="1"/>
@@ -4334,7 +3908,7 @@
       <c r="S146" s="1"/>
       <c r="T146" s="1"/>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="147">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="1"/>
@@ -4356,7 +3930,7 @@
       <c r="S147" s="1"/>
       <c r="T147" s="1"/>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="148">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="1"/>
@@ -4378,7 +3952,7 @@
       <c r="S148" s="1"/>
       <c r="T148" s="1"/>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="149">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="1"/>
@@ -4400,7 +3974,7 @@
       <c r="S149" s="1"/>
       <c r="T149" s="1"/>
     </row>
-    <row r="150" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="150">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="1"/>
@@ -4422,7 +3996,7 @@
       <c r="S150" s="1"/>
       <c r="T150" s="1"/>
     </row>
-    <row r="151" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="151">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="1"/>
@@ -4444,7 +4018,7 @@
       <c r="S151" s="1"/>
       <c r="T151" s="1"/>
     </row>
-    <row r="152" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="152">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="1"/>
@@ -4466,7 +4040,7 @@
       <c r="S152" s="1"/>
       <c r="T152" s="1"/>
     </row>
-    <row r="153" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="153">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="1"/>
@@ -4488,7 +4062,7 @@
       <c r="S153" s="1"/>
       <c r="T153" s="1"/>
     </row>
-    <row r="154" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="154">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="1"/>
@@ -4510,7 +4084,7 @@
       <c r="S154" s="1"/>
       <c r="T154" s="1"/>
     </row>
-    <row r="155" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="155">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="1"/>
@@ -4532,7 +4106,7 @@
       <c r="S155" s="1"/>
       <c r="T155" s="1"/>
     </row>
-    <row r="156" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="156">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="1"/>
@@ -4554,7 +4128,7 @@
       <c r="S156" s="1"/>
       <c r="T156" s="1"/>
     </row>
-    <row r="157" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="157">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="1"/>
@@ -4576,7 +4150,7 @@
       <c r="S157" s="1"/>
       <c r="T157" s="1"/>
     </row>
-    <row r="158" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="158">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="1"/>
@@ -4598,7 +4172,7 @@
       <c r="S158" s="1"/>
       <c r="T158" s="1"/>
     </row>
-    <row r="159" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="159">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="1"/>
@@ -4620,7 +4194,7 @@
       <c r="S159" s="1"/>
       <c r="T159" s="1"/>
     </row>
-    <row r="160" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="160">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="1"/>
@@ -4642,7 +4216,7 @@
       <c r="S160" s="1"/>
       <c r="T160" s="1"/>
     </row>
-    <row r="161" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="161">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="1"/>
@@ -4664,7 +4238,7 @@
       <c r="S161" s="1"/>
       <c r="T161" s="1"/>
     </row>
-    <row r="162" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="162">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="1"/>
@@ -4686,7 +4260,7 @@
       <c r="S162" s="1"/>
       <c r="T162" s="1"/>
     </row>
-    <row r="163" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="163">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="1"/>
@@ -4708,7 +4282,7 @@
       <c r="S163" s="1"/>
       <c r="T163" s="1"/>
     </row>
-    <row r="164" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="164">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="1"/>
@@ -4730,7 +4304,7 @@
       <c r="S164" s="1"/>
       <c r="T164" s="1"/>
     </row>
-    <row r="165" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="165">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="1"/>
@@ -4752,7 +4326,7 @@
       <c r="S165" s="1"/>
       <c r="T165" s="1"/>
     </row>
-    <row r="166" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="166">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="1"/>
@@ -4774,7 +4348,7 @@
       <c r="S166" s="1"/>
       <c r="T166" s="1"/>
     </row>
-    <row r="167" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="167">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="1"/>
@@ -4796,7 +4370,7 @@
       <c r="S167" s="1"/>
       <c r="T167" s="1"/>
     </row>
-    <row r="168" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="168">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="1"/>
@@ -4818,7 +4392,7 @@
       <c r="S168" s="1"/>
       <c r="T168" s="1"/>
     </row>
-    <row r="169" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="169">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="1"/>
@@ -4840,7 +4414,7 @@
       <c r="S169" s="1"/>
       <c r="T169" s="1"/>
     </row>
-    <row r="170" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="170">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="1"/>
@@ -4862,7 +4436,7 @@
       <c r="S170" s="1"/>
       <c r="T170" s="1"/>
     </row>
-    <row r="171" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="171">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="1"/>
@@ -4884,7 +4458,7 @@
       <c r="S171" s="1"/>
       <c r="T171" s="1"/>
     </row>
-    <row r="172" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="172">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="1"/>
@@ -4906,7 +4480,7 @@
       <c r="S172" s="1"/>
       <c r="T172" s="1"/>
     </row>
-    <row r="173" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="173">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="1"/>
@@ -4928,7 +4502,7 @@
       <c r="S173" s="1"/>
       <c r="T173" s="1"/>
     </row>
-    <row r="174" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="174">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="1"/>
@@ -4950,7 +4524,7 @@
       <c r="S174" s="1"/>
       <c r="T174" s="1"/>
     </row>
-    <row r="175" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="175">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="1"/>
@@ -4972,7 +4546,7 @@
       <c r="S175" s="1"/>
       <c r="T175" s="1"/>
     </row>
-    <row r="176" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="176">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="1"/>
@@ -4994,7 +4568,7 @@
       <c r="S176" s="1"/>
       <c r="T176" s="1"/>
     </row>
-    <row r="177" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="177">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="1"/>
@@ -5016,7 +4590,7 @@
       <c r="S177" s="1"/>
       <c r="T177" s="1"/>
     </row>
-    <row r="178" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="178">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="1"/>
@@ -5038,7 +4612,7 @@
       <c r="S178" s="1"/>
       <c r="T178" s="1"/>
     </row>
-    <row r="179" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="179">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="1"/>
@@ -5060,7 +4634,7 @@
       <c r="S179" s="1"/>
       <c r="T179" s="1"/>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="180">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="1"/>
@@ -5082,7 +4656,7 @@
       <c r="S180" s="1"/>
       <c r="T180" s="1"/>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="181">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="1"/>
@@ -5104,7 +4678,7 @@
       <c r="S181" s="1"/>
       <c r="T181" s="1"/>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="182">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="1"/>
@@ -5126,7 +4700,7 @@
       <c r="S182" s="1"/>
       <c r="T182" s="1"/>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="183">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="1"/>
@@ -5148,7 +4722,7 @@
       <c r="S183" s="1"/>
       <c r="T183" s="1"/>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="184">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="1"/>
@@ -5170,7 +4744,7 @@
       <c r="S184" s="1"/>
       <c r="T184" s="1"/>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="185">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="1"/>
@@ -5192,7 +4766,7 @@
       <c r="S185" s="1"/>
       <c r="T185" s="1"/>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="186">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="1"/>
@@ -5214,7 +4788,7 @@
       <c r="S186" s="1"/>
       <c r="T186" s="1"/>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="187">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="1"/>
@@ -5236,7 +4810,7 @@
       <c r="S187" s="1"/>
       <c r="T187" s="1"/>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="188">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="1"/>
@@ -5258,7 +4832,7 @@
       <c r="S188" s="1"/>
       <c r="T188" s="1"/>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="189">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="1"/>
@@ -5280,7 +4854,7 @@
       <c r="S189" s="1"/>
       <c r="T189" s="1"/>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="190">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="1"/>
@@ -5302,7 +4876,7 @@
       <c r="S190" s="1"/>
       <c r="T190" s="1"/>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="191">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="1"/>
@@ -5324,7 +4898,7 @@
       <c r="S191" s="1"/>
       <c r="T191" s="1"/>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="192">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
       <c r="C192" s="1"/>
@@ -5346,7 +4920,7 @@
       <c r="S192" s="1"/>
       <c r="T192" s="1"/>
     </row>
-    <row r="193" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="193">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="1"/>
@@ -5368,7 +4942,7 @@
       <c r="S193" s="1"/>
       <c r="T193" s="1"/>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="194">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
       <c r="C194" s="1"/>
@@ -5390,7 +4964,7 @@
       <c r="S194" s="1"/>
       <c r="T194" s="1"/>
     </row>
-    <row r="195" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="195">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
       <c r="C195" s="1"/>
@@ -5412,7 +4986,7 @@
       <c r="S195" s="1"/>
       <c r="T195" s="1"/>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="196">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="1"/>
@@ -5434,7 +5008,7 @@
       <c r="S196" s="1"/>
       <c r="T196" s="1"/>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="197">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
       <c r="C197" s="1"/>
@@ -5456,7 +5030,7 @@
       <c r="S197" s="1"/>
       <c r="T197" s="1"/>
     </row>
-    <row r="198" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="198">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="1"/>
@@ -5478,7 +5052,7 @@
       <c r="S198" s="1"/>
       <c r="T198" s="1"/>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="199">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
       <c r="C199" s="1"/>
@@ -5500,30 +5074,7 @@
       <c r="S199" s="1"/>
       <c r="T199" s="1"/>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A200" s="2"/>
-      <c r="B200" s="2"/>
-      <c r="C200" s="1"/>
-      <c r="D200" s="1"/>
-      <c r="E200" s="1"/>
-      <c r="F200" s="1"/>
-      <c r="G200" s="1"/>
-      <c r="H200" s="1"/>
-      <c r="I200" s="1"/>
-      <c r="J200" s="1"/>
-      <c r="K200" s="1"/>
-      <c r="L200" s="1"/>
-      <c r="M200" s="1"/>
-      <c r="N200" s="1"/>
-      <c r="O200" s="1"/>
-      <c r="P200" s="1"/>
-      <c r="Q200" s="1"/>
-      <c r="R200" s="1"/>
-      <c r="S200" s="1"/>
-      <c r="T200" s="1"/>
-    </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>